<commit_message>
Atualizar planilhas de dados de clientes e base instalada
</commit_message>
<xml_diff>
--- a/data/clientes.xlsx
+++ b/data/clientes.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://maquinascomprint-my.sharepoint.com/personal/ricardo_almeida_comprint_com_br/Documents/PROJETOS/OUTROS/Programação/chatbot-whatsapp-estoque/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="337" documentId="11_FFC65FC0F879EECECE170B54ABAE8EF57AB2EA2D" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E1005F7F-8A94-4540-AE6B-7C95C4BD8E9D}"/>
+  <xr:revisionPtr revIDLastSave="339" documentId="11_FFC65FC0F879EECECE170B54ABAE8EF57AB2EA2D" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6E05A0BF-C769-4817-B2D3-25222AC3E4C5}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="228" uniqueCount="161">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="229" uniqueCount="161">
   <si>
     <t>CLIENTE</t>
   </si>
@@ -884,13 +884,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:F95"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="23.140625" customWidth="1"/>
-    <col min="2" max="6" width="25.5703125" customWidth="1"/>
+    <col min="1" max="1" width="23.1796875" customWidth="1"/>
+    <col min="2" max="6" width="25.54296875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -910,7 +910,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -918,7 +918,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>2</v>
       </c>
@@ -932,7 +932,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -943,7 +943,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>4</v>
       </c>
@@ -951,7 +951,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>5</v>
       </c>
@@ -959,7 +959,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>6</v>
       </c>
@@ -967,7 +967,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>7</v>
       </c>
@@ -975,7 +975,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>92</v>
       </c>
@@ -983,7 +983,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>8</v>
       </c>
@@ -994,7 +994,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>9</v>
       </c>
@@ -1002,7 +1002,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>10</v>
       </c>
@@ -1013,7 +1013,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>11</v>
       </c>
@@ -1027,7 +1027,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>35</v>
       </c>
@@ -1035,7 +1035,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>12</v>
       </c>
@@ -1046,7 +1046,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>13</v>
       </c>
@@ -1054,7 +1054,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>14</v>
       </c>
@@ -1062,7 +1062,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>15</v>
       </c>
@@ -1073,7 +1073,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>16</v>
       </c>
@@ -1081,7 +1081,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>17</v>
       </c>
@@ -1089,7 +1089,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>18</v>
       </c>
@@ -1103,7 +1103,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>90</v>
       </c>
@@ -1111,7 +1111,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>19</v>
       </c>
@@ -1119,7 +1119,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>20</v>
       </c>
@@ -1127,7 +1127,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>21</v>
       </c>
@@ -1140,8 +1140,11 @@
       <c r="D25" t="s">
         <v>96</v>
       </c>
-    </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E25" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>22</v>
       </c>
@@ -1152,7 +1155,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>93</v>
       </c>
@@ -1160,7 +1163,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>23</v>
       </c>
@@ -1168,7 +1171,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>24</v>
       </c>
@@ -1176,7 +1179,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>25</v>
       </c>
@@ -1187,7 +1190,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>26</v>
       </c>
@@ -1195,7 +1198,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>27</v>
       </c>
@@ -1206,7 +1209,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>28</v>
       </c>
@@ -1214,7 +1217,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>29</v>
       </c>
@@ -1222,7 +1225,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>30</v>
       </c>
@@ -1233,7 +1236,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>31</v>
       </c>
@@ -1244,7 +1247,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>32</v>
       </c>
@@ -1252,7 +1255,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
         <v>33</v>
       </c>
@@ -1263,7 +1266,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
         <v>34</v>
       </c>
@@ -1277,7 +1280,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
         <v>36</v>
       </c>
@@ -1288,7 +1291,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
         <v>37</v>
       </c>
@@ -1296,7 +1299,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
         <v>38</v>
       </c>
@@ -1307,7 +1310,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
         <v>39</v>
       </c>
@@ -1315,7 +1318,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
         <v>40</v>
       </c>
@@ -1323,7 +1326,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
         <v>41</v>
       </c>
@@ -1331,7 +1334,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
         <v>42</v>
       </c>
@@ -1339,7 +1342,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
         <v>43</v>
       </c>
@@ -1350,7 +1353,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
         <v>94</v>
       </c>
@@ -1358,7 +1361,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
         <v>44</v>
       </c>
@@ -1369,7 +1372,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
         <v>45</v>
       </c>
@@ -1377,7 +1380,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
         <v>46</v>
       </c>
@@ -1385,7 +1388,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
         <v>47</v>
       </c>
@@ -1396,7 +1399,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="53" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
         <v>48</v>
       </c>
@@ -1404,7 +1407,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="54" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
         <v>49</v>
       </c>
@@ -1412,7 +1415,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="55" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
         <v>50</v>
       </c>
@@ -1420,7 +1423,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="56" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A56" t="s">
         <v>51</v>
       </c>
@@ -1428,7 +1431,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="57" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A57" t="s">
         <v>95</v>
       </c>
@@ -1436,7 +1439,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="58" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A58" t="s">
         <v>52</v>
       </c>
@@ -1444,7 +1447,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="59" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A59" t="s">
         <v>53</v>
       </c>
@@ -1452,7 +1455,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="60" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A60" t="s">
         <v>144</v>
       </c>
@@ -1460,7 +1463,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="61" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A61" t="s">
         <v>54</v>
       </c>
@@ -1471,7 +1474,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="62" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A62" t="s">
         <v>55</v>
       </c>
@@ -1479,7 +1482,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="63" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A63" t="s">
         <v>56</v>
       </c>
@@ -1490,7 +1493,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="64" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A64" t="s">
         <v>57</v>
       </c>
@@ -1498,7 +1501,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="65" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A65" t="s">
         <v>58</v>
       </c>
@@ -1506,7 +1509,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="66" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A66" t="s">
         <v>91</v>
       </c>
@@ -1514,7 +1517,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="67" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A67" t="s">
         <v>19</v>
       </c>
@@ -1522,7 +1525,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="68" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A68" t="s">
         <v>59</v>
       </c>
@@ -1530,7 +1533,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="69" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A69" t="s">
         <v>60</v>
       </c>
@@ -1538,7 +1541,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="70" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A70" t="s">
         <v>61</v>
       </c>
@@ -1546,7 +1549,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="71" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A71" t="s">
         <v>62</v>
       </c>
@@ -1554,7 +1557,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="72" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A72" t="s">
         <v>63</v>
       </c>
@@ -1562,7 +1565,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="73" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A73" t="s">
         <v>64</v>
       </c>
@@ -1573,7 +1576,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="74" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A74" t="s">
         <v>65</v>
       </c>
@@ -1581,7 +1584,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="75" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A75" t="s">
         <v>66</v>
       </c>
@@ -1589,7 +1592,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="76" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A76" t="s">
         <v>67</v>
       </c>
@@ -1597,7 +1600,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="77" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A77" t="s">
         <v>68</v>
       </c>
@@ -1605,7 +1608,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="78" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A78" t="s">
         <v>69</v>
       </c>
@@ -1616,7 +1619,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="79" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A79" t="s">
         <v>70</v>
       </c>
@@ -1627,7 +1630,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="80" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A80" t="s">
         <v>71</v>
       </c>
@@ -1638,7 +1641,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="81" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A81" t="s">
         <v>72</v>
       </c>
@@ -1646,7 +1649,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="82" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A82" t="s">
         <v>73</v>
       </c>
@@ -1654,7 +1657,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="83" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A83" t="s">
         <v>74</v>
       </c>
@@ -1662,7 +1665,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="84" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A84" t="s">
         <v>75</v>
       </c>
@@ -1676,7 +1679,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="85" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A85" t="s">
         <v>76</v>
       </c>
@@ -1684,7 +1687,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="86" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A86" t="s">
         <v>77</v>
       </c>
@@ -1692,7 +1695,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="87" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A87" t="s">
         <v>78</v>
       </c>
@@ -1700,7 +1703,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="88" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A88" t="s">
         <v>79</v>
       </c>
@@ -1708,7 +1711,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="89" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A89" t="s">
         <v>80</v>
       </c>
@@ -1716,7 +1719,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="90" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A90" t="s">
         <v>81</v>
       </c>
@@ -1724,7 +1727,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="91" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A91" t="s">
         <v>82</v>
       </c>
@@ -1732,7 +1735,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="92" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A92" t="s">
         <v>83</v>
       </c>
@@ -1740,7 +1743,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="93" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A93" t="s">
         <v>84</v>
       </c>
@@ -1748,7 +1751,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="94" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A94" t="s">
         <v>156</v>
       </c>
@@ -1756,7 +1759,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="95" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A95" t="s">
         <v>158</v>
       </c>

</xml_diff>

<commit_message>
Update data files and add Comprint CSSP reports
</commit_message>
<xml_diff>
--- a/data/clientes.xlsx
+++ b/data/clientes.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://maquinascomprint-my.sharepoint.com/personal/ricardo_almeida_comprint_com_br/Documents/PROJETOS/OUTROS/Programação/chatbot-whatsapp-estoque/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="340" documentId="11_FFC65FC0F879EECECE170B54ABAE8EF57AB2EA2D" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D7EF1D17-8860-4C4E-99CF-44E04B5B793D}"/>
+  <xr:revisionPtr revIDLastSave="342" documentId="11_FFC65FC0F879EECECE170B54ABAE8EF57AB2EA2D" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{39462ADE-C498-4FA5-8D5D-D854CEDCC443}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="230" uniqueCount="161">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="232" uniqueCount="162">
   <si>
     <t>CLIENTE</t>
   </si>
@@ -516,6 +516,9 @@
   </si>
   <si>
     <t>ABG DS3 - VENDA</t>
+  </si>
+  <si>
+    <t>DELPAK</t>
   </si>
 </sst>
 </file>
@@ -883,7 +886,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F95"/>
+  <dimension ref="A1:F96"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="23.1796875" customWidth="1"/>
@@ -1770,6 +1773,14 @@
         <v>159</v>
       </c>
     </row>
+    <row r="96" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A96" t="s">
+        <v>161</v>
+      </c>
+      <c r="B96" t="s">
+        <v>102</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>